<commit_message>
PAUSED: checkpoint, writers open
Continues 882c2c1.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task192/golden/boletim_vigilancia_2026S2.xlsx
+++ b/task192/golden/boletim_vigilancia_2026S2.xlsx
@@ -97,7 +97,7 @@
     <t>Municipios tocados</t>
   </si>
   <si>
-    <t>Quota da rede de parceiros, %</t>
+    <t>Acoes relatadas pela rede de parceiros</t>
   </si>
   <si>
     <t>Q1</t>
@@ -217,7 +217,7 @@
     <t>2026-10-30</t>
   </si>
   <si>
-    <t>Uma acao e um tema numa localidade num dia, qualquer que seja o numero de relatos. A quota e a parte das acoes da quinzena que a rede de parceiros relatou. As quinzenas tem catorze dias e a ultima tem quinze.</t>
+    <t>Uma acao e um tema numa localidade num dia, qualquer que seja o numero de relatos. A ultima coluna conta as acoes da quinzena de que a rede de parceiros entregou relato, cada acao uma vez. As quinzenas tem catorze dias e a ultima tem quinze.</t>
   </si>
   <si>
     <t>Relatos por via de acesso no periodo</t>
@@ -889,7 +889,7 @@
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -933,8 +933,8 @@
       <c r="E4" s="12">
         <v>111</v>
       </c>
-      <c r="F4" s="13">
-        <v>23.9</v>
+      <c r="F4" s="12">
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -953,8 +953,8 @@
       <c r="E5" s="12">
         <v>110</v>
       </c>
-      <c r="F5" s="13">
-        <v>26.5</v>
+      <c r="F5" s="12">
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -973,8 +973,8 @@
       <c r="E6" s="12">
         <v>100</v>
       </c>
-      <c r="F6" s="13">
-        <v>20.9</v>
+      <c r="F6" s="12">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -993,8 +993,8 @@
       <c r="E7" s="12">
         <v>103</v>
       </c>
-      <c r="F7" s="13">
-        <v>20.2</v>
+      <c r="F7" s="12">
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1013,8 +1013,8 @@
       <c r="E8" s="12">
         <v>104</v>
       </c>
-      <c r="F8" s="13">
-        <v>25.3</v>
+      <c r="F8" s="12">
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1033,8 +1033,8 @@
       <c r="E9" s="12">
         <v>103</v>
       </c>
-      <c r="F9" s="13">
-        <v>23.6</v>
+      <c r="F9" s="12">
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1053,8 +1053,8 @@
       <c r="E10" s="12">
         <v>100</v>
       </c>
-      <c r="F10" s="13">
-        <v>27.8</v>
+      <c r="F10" s="12">
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1073,8 +1073,8 @@
       <c r="E11" s="12">
         <v>105</v>
       </c>
-      <c r="F11" s="13">
-        <v>25.5</v>
+      <c r="F11" s="12">
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1093,8 +1093,8 @@
       <c r="E12" s="12">
         <v>111</v>
       </c>
-      <c r="F12" s="13">
-        <v>23.4</v>
+      <c r="F12" s="12">
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1113,8 +1113,8 @@
       <c r="E13" s="12">
         <v>116</v>
       </c>
-      <c r="F13" s="13">
-        <v>24.8</v>
+      <c r="F13" s="12">
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1133,8 +1133,8 @@
       <c r="E14" s="12">
         <v>118</v>
       </c>
-      <c r="F14" s="13">
-        <v>26.5</v>
+      <c r="F14" s="12">
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1153,8 +1153,8 @@
       <c r="E15" s="12">
         <v>119</v>
       </c>
-      <c r="F15" s="13">
-        <v>26.4</v>
+      <c r="F15" s="12">
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1173,8 +1173,8 @@
       <c r="E16" s="12">
         <v>119</v>
       </c>
-      <c r="F16" s="13">
-        <v>25.4</v>
+      <c r="F16" s="12">
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -1419,7 +1419,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="12">
-        <v>732</v>
+        <v>726</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>